<commit_message>
feat: add shared item data table, inventory services, procurement pipelines, and purchase management UI pages
</commit_message>
<xml_diff>
--- a/data/san_pham_mau.xlsx
+++ b/data/san_pham_mau.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\smart-erp\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Do_an_lien_nganh\smart-erp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E85BF774-1013-4B7E-B685-6161B8728D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1652E678-AE66-4232-945B-6EBCE772BC8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16354" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SanPham" sheetId="1" r:id="rId1"/>
     <sheet name="ThongKe" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SanPham!$A$1:$G$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SanPham!$A$1:$H$101</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="447">
   <si>
     <t>sku</t>
   </si>
@@ -1335,13 +1335,43 @@
   </si>
   <si>
     <t>gross price</t>
+  </si>
+  <si>
+    <t>com</t>
+  </si>
+  <si>
+    <t>Hàn Quốc</t>
+  </si>
+  <si>
+    <t>Nhật Bản</t>
+  </si>
+  <si>
+    <t>Việt Nam</t>
+  </si>
+  <si>
+    <t>Thái Lan</t>
+  </si>
+  <si>
+    <t>Trung Quốc</t>
+  </si>
+  <si>
+    <t>Đức</t>
+  </si>
+  <si>
+    <t>Anh</t>
+  </si>
+  <si>
+    <t>Hà Lan</t>
+  </si>
+  <si>
+    <t>Mỹ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1358,6 +1388,11 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1385,7 +1420,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1393,6 +1428,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1695,19 +1734,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G101"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:H101"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="70" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1721,16 +1761,19 @@
         <v>435</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -1744,16 +1787,19 @@
         <v>7</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="3">
+      <c r="G2" s="3">
         <v>11800000</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1766,17 +1812,20 @@
       <c r="D3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="3">
+      <c r="G3" s="3">
         <v>7900000</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
@@ -1789,17 +1838,20 @@
       <c r="D4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="3">
+      <c r="G4" s="3">
         <v>14500000</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1812,17 +1864,20 @@
       <c r="D5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="3">
+      <c r="G5" s="3">
         <v>17900000</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
@@ -1835,17 +1890,20 @@
       <c r="D6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="3">
+      <c r="G6" s="3">
         <v>14900000</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>29</v>
       </c>
@@ -1858,17 +1916,20 @@
       <c r="D7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="3">
+      <c r="G7" s="3">
         <v>6800000</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>33</v>
       </c>
@@ -1881,17 +1942,20 @@
       <c r="D8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="3">
+      <c r="G8" s="3">
         <v>22800000</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>37</v>
       </c>
@@ -1904,17 +1968,20 @@
       <c r="D9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="3">
+      <c r="G9" s="3">
         <v>9000000</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>41</v>
       </c>
@@ -1927,17 +1994,20 @@
       <c r="D10" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="6" t="s">
+        <v>439</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F10" s="3">
+      <c r="G10" s="3">
         <v>9700000</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>45</v>
       </c>
@@ -1950,17 +2020,20 @@
       <c r="D11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="3">
+      <c r="G11" s="3">
         <v>17400000</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>50</v>
       </c>
@@ -1973,17 +2046,20 @@
       <c r="D12" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F12" s="3">
+      <c r="G12" s="3">
         <v>17900000</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>55</v>
       </c>
@@ -1996,17 +2072,20 @@
       <c r="D13" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F13" s="3">
+      <c r="G13" s="3">
         <v>4900000</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="H13" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>60</v>
       </c>
@@ -2019,17 +2098,20 @@
       <c r="D14" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F14" s="3">
+      <c r="G14" s="3">
         <v>22600000</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="H14" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>64</v>
       </c>
@@ -2042,17 +2124,20 @@
       <c r="D15" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F15" s="3">
+      <c r="G15" s="3">
         <v>4500000</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>68</v>
       </c>
@@ -2065,17 +2150,20 @@
       <c r="D16" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F16" s="3">
+      <c r="G16" s="3">
         <v>14500000</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="H16" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>71</v>
       </c>
@@ -2088,17 +2176,20 @@
       <c r="D17" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F17" s="3">
+      <c r="G17" s="3">
         <v>14700000</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="H17" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>77</v>
       </c>
@@ -2111,17 +2202,20 @@
       <c r="D18" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F18" s="3">
+      <c r="G18" s="3">
         <v>14900000</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="H18" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>81</v>
       </c>
@@ -2134,17 +2228,20 @@
       <c r="D19" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F19" s="3">
+      <c r="G19" s="3">
         <v>15300000</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>85</v>
       </c>
@@ -2157,17 +2254,20 @@
       <c r="D20" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F20" s="3">
+      <c r="G20" s="3">
         <v>15000000</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="H20" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>90</v>
       </c>
@@ -2180,17 +2280,20 @@
       <c r="D21" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F21" s="3">
+      <c r="G21" s="3">
         <v>14900000</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="H21" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>94</v>
       </c>
@@ -2203,17 +2306,20 @@
       <c r="D22" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F22" s="3">
+      <c r="G22" s="3">
         <v>13400000</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="H22" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>98</v>
       </c>
@@ -2226,17 +2332,20 @@
       <c r="D23" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F23" s="3">
+      <c r="G23" s="3">
         <v>9200000</v>
       </c>
-      <c r="G23" s="2" t="s">
+      <c r="H23" s="2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>102</v>
       </c>
@@ -2249,17 +2358,20 @@
       <c r="D24" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F24" s="3">
+      <c r="G24" s="3">
         <v>8500000</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="H24" s="2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>106</v>
       </c>
@@ -2272,17 +2384,20 @@
       <c r="D25" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F25" s="3">
+      <c r="G25" s="3">
         <v>13500000</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="H25" s="2" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>110</v>
       </c>
@@ -2295,17 +2410,20 @@
       <c r="D26" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F26" s="3">
+      <c r="G26" s="3">
         <v>13000000</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="H26" s="2" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>114</v>
       </c>
@@ -2318,17 +2436,20 @@
       <c r="D27" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="3">
+      <c r="G27" s="3">
         <v>11100000</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="H27" s="2" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>118</v>
       </c>
@@ -2341,17 +2462,20 @@
       <c r="D28" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F28" s="3">
+      <c r="G28" s="3">
         <v>11400000</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="H28" s="2" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>122</v>
       </c>
@@ -2364,17 +2488,20 @@
       <c r="D29" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="E29" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F29" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F29" s="3">
+      <c r="G29" s="3">
         <v>14900000</v>
       </c>
-      <c r="G29" s="2" t="s">
+      <c r="H29" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>125</v>
       </c>
@@ -2387,17 +2514,20 @@
       <c r="D30" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E30" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F30" s="3">
+      <c r="G30" s="3">
         <v>10700000</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="H30" s="2" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>129</v>
       </c>
@@ -2410,17 +2540,20 @@
       <c r="D31" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="E31" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F31" s="3">
+      <c r="G31" s="3">
         <v>14700000</v>
       </c>
-      <c r="G31" s="2" t="s">
+      <c r="H31" s="2" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>133</v>
       </c>
@@ -2433,17 +2566,20 @@
       <c r="D32" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E32" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F32" s="3">
+      <c r="G32" s="3">
         <v>9400000</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="H32" s="2" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>138</v>
       </c>
@@ -2456,17 +2592,20 @@
       <c r="D33" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F33" s="3">
+      <c r="G33" s="3">
         <v>9600000</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="H33" s="2" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>142</v>
       </c>
@@ -2479,17 +2618,20 @@
       <c r="D34" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="E34" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F34" s="3">
+      <c r="G34" s="3">
         <v>8500000</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="H34" s="2" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>146</v>
       </c>
@@ -2502,17 +2644,20 @@
       <c r="D35" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="E35" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F35" s="3">
+      <c r="G35" s="3">
         <v>17800000</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="H35" s="2" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>151</v>
       </c>
@@ -2525,17 +2670,20 @@
       <c r="D36" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="E36" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F36" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F36" s="3">
+      <c r="G36" s="3">
         <v>14800000</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="H36" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>155</v>
       </c>
@@ -2548,17 +2696,20 @@
       <c r="D37" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="E37" t="s">
+        <v>439</v>
+      </c>
+      <c r="F37" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F37" s="3">
+      <c r="G37" s="3">
         <v>12200000</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="H37" s="2" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>160</v>
       </c>
@@ -2571,17 +2722,20 @@
       <c r="D38" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="E38" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F38" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F38" s="3">
+      <c r="G38" s="3">
         <v>8400000</v>
       </c>
-      <c r="G38" s="2" t="s">
+      <c r="H38" s="2" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>164</v>
       </c>
@@ -2594,17 +2748,20 @@
       <c r="D39" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E39" s="2" t="s">
+      <c r="E39" t="s">
+        <v>439</v>
+      </c>
+      <c r="F39" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F39" s="3">
+      <c r="G39" s="3">
         <v>17100000</v>
       </c>
-      <c r="G39" s="2" t="s">
+      <c r="H39" s="2" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>167</v>
       </c>
@@ -2617,17 +2774,20 @@
       <c r="D40" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="E40" s="2" t="s">
+      <c r="E40" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F40" s="3">
+      <c r="G40" s="3">
         <v>14300000</v>
       </c>
-      <c r="G40" s="2" t="s">
+      <c r="H40" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>172</v>
       </c>
@@ -2640,17 +2800,20 @@
       <c r="D41" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="E41" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F41" s="3">
+      <c r="G41" s="3">
         <v>12300000</v>
       </c>
-      <c r="G41" s="2" t="s">
+      <c r="H41" s="2" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>176</v>
       </c>
@@ -2663,17 +2826,20 @@
       <c r="D42" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E42" s="2" t="s">
+      <c r="E42" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F42" s="3">
+      <c r="G42" s="3">
         <v>11900000</v>
       </c>
-      <c r="G42" s="2" t="s">
+      <c r="H42" s="2" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>180</v>
       </c>
@@ -2686,17 +2852,20 @@
       <c r="D43" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="E43" s="2" t="s">
+      <c r="E43" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F43" s="3">
+      <c r="G43" s="3">
         <v>12500000</v>
       </c>
-      <c r="G43" s="2" t="s">
+      <c r="H43" s="2" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>184</v>
       </c>
@@ -2709,17 +2878,20 @@
       <c r="D44" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="E44" s="2" t="s">
+      <c r="E44" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F44" s="3">
+      <c r="G44" s="3">
         <v>9400000</v>
       </c>
-      <c r="G44" s="2" t="s">
+      <c r="H44" s="2" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>188</v>
       </c>
@@ -2732,17 +2904,20 @@
       <c r="D45" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="E45" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F45" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F45" s="3">
+      <c r="G45" s="3">
         <v>6300000</v>
       </c>
-      <c r="G45" s="2" t="s">
+      <c r="H45" s="2" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>192</v>
       </c>
@@ -2755,17 +2930,20 @@
       <c r="D46" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="E46" s="2" t="s">
+      <c r="E46" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F46" s="3">
+      <c r="G46" s="3">
         <v>9000000</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="H46" s="2" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>196</v>
       </c>
@@ -2778,17 +2956,20 @@
       <c r="D47" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="E47" s="2" t="s">
+      <c r="E47" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F47" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F47" s="3">
+      <c r="G47" s="3">
         <v>15800000</v>
       </c>
-      <c r="G47" s="2" t="s">
+      <c r="H47" s="2" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>200</v>
       </c>
@@ -2801,40 +2982,46 @@
       <c r="D48" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="E48" s="2" t="s">
+      <c r="E48" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F48" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F48" s="3">
+      <c r="G48" s="3">
         <v>15000000</v>
       </c>
-      <c r="G48" s="2" t="s">
+      <c r="H48" s="2" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>204</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="C49" s="5" t="s">
         <v>87</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="E49" s="2" t="s">
+      <c r="E49" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F49" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F49" s="3">
+      <c r="G49" s="3">
         <v>9000000</v>
       </c>
-      <c r="G49" s="2" t="s">
+      <c r="H49" s="2" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>208</v>
       </c>
@@ -2847,17 +3034,20 @@
       <c r="D50" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="E50" s="2" t="s">
+      <c r="E50" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F50" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F50" s="3">
+      <c r="G50" s="3">
         <v>14500000</v>
       </c>
-      <c r="G50" s="2" t="s">
+      <c r="H50" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>211</v>
       </c>
@@ -2870,17 +3060,20 @@
       <c r="D51" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="E51" s="2" t="s">
+      <c r="E51" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F51" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F51" s="3">
+      <c r="G51" s="3">
         <v>9700000</v>
       </c>
-      <c r="G51" s="2" t="s">
+      <c r="H51" s="2" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>215</v>
       </c>
@@ -2893,17 +3086,20 @@
       <c r="D52" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="E52" s="2" t="s">
+      <c r="E52" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F52" s="3">
+      <c r="G52" s="3">
         <v>16000000</v>
       </c>
-      <c r="G52" s="2" t="s">
+      <c r="H52" s="2" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>220</v>
       </c>
@@ -2916,17 +3112,20 @@
       <c r="D53" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="E53" s="2" t="s">
+      <c r="E53" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="F53" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F53" s="3">
+      <c r="G53" s="3">
         <v>15000000</v>
       </c>
-      <c r="G53" s="2" t="s">
+      <c r="H53" s="2" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>225</v>
       </c>
@@ -2939,17 +3138,20 @@
       <c r="D54" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="E54" s="2" t="s">
+      <c r="E54" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="F54" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F54" s="3">
+      <c r="G54" s="3">
         <v>14000000</v>
       </c>
-      <c r="G54" s="2" t="s">
+      <c r="H54" s="2" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>229</v>
       </c>
@@ -2962,17 +3164,20 @@
       <c r="D55" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="E55" s="2" t="s">
+      <c r="E55" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F55" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F55" s="3">
+      <c r="G55" s="3">
         <v>14000000</v>
       </c>
-      <c r="G55" s="2" t="s">
+      <c r="H55" s="2" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>233</v>
       </c>
@@ -2985,17 +3190,20 @@
       <c r="D56" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="E56" s="2" t="s">
+      <c r="E56" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F56" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F56" s="3">
+      <c r="G56" s="3">
         <v>17000000</v>
       </c>
-      <c r="G56" s="2" t="s">
+      <c r="H56" s="2" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>237</v>
       </c>
@@ -3008,17 +3216,20 @@
       <c r="D57" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="E57" s="2" t="s">
+      <c r="E57" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F57" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F57" s="3">
+      <c r="G57" s="3">
         <v>13000000</v>
       </c>
-      <c r="G57" s="2" t="s">
+      <c r="H57" s="2" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>241</v>
       </c>
@@ -3031,17 +3242,20 @@
       <c r="D58" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="E58" s="2" t="s">
+      <c r="E58" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F58" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F58" s="3">
+      <c r="G58" s="3">
         <v>16000000</v>
       </c>
-      <c r="G58" s="2" t="s">
+      <c r="H58" s="2" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>245</v>
       </c>
@@ -3054,17 +3268,20 @@
       <c r="D59" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="E59" s="2" t="s">
+      <c r="E59" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F59" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F59" s="3">
+      <c r="G59" s="3">
         <v>15000000</v>
       </c>
-      <c r="G59" s="2" t="s">
+      <c r="H59" s="2" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>249</v>
       </c>
@@ -3077,17 +3294,20 @@
       <c r="D60" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="E60" s="2" t="s">
+      <c r="E60" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F60" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F60" s="3">
+      <c r="G60" s="3">
         <v>18000000</v>
       </c>
-      <c r="G60" s="2" t="s">
+      <c r="H60" s="2" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>253</v>
       </c>
@@ -3100,17 +3320,20 @@
       <c r="D61" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="E61" s="2" t="s">
+      <c r="E61" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F61" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F61" s="3">
+      <c r="G61" s="3">
         <v>14000000</v>
       </c>
-      <c r="G61" s="2" t="s">
+      <c r="H61" s="2" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>257</v>
       </c>
@@ -3123,17 +3346,20 @@
       <c r="D62" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="E62" s="2" t="s">
+      <c r="E62" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="F62" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F62" s="3">
+      <c r="G62" s="3">
         <v>4700000</v>
       </c>
-      <c r="G62" s="2" t="s">
+      <c r="H62" s="2" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>263</v>
       </c>
@@ -3146,17 +3372,20 @@
       <c r="D63" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="E63" s="2" t="s">
+      <c r="E63" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F63" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F63" s="3">
+      <c r="G63" s="3">
         <v>4000000</v>
       </c>
-      <c r="G63" s="2" t="s">
+      <c r="H63" s="2" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>267</v>
       </c>
@@ -3169,17 +3398,20 @@
       <c r="D64" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="E64" s="2" t="s">
+      <c r="E64" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F64" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F64" s="3">
+      <c r="G64" s="3">
         <v>3900000</v>
       </c>
-      <c r="G64" s="2" t="s">
+      <c r="H64" s="2" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>271</v>
       </c>
@@ -3192,63 +3424,72 @@
       <c r="D65" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="E65" s="2" t="s">
+      <c r="E65" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F65" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F65" s="3">
+      <c r="G65" s="3">
         <v>7500000</v>
       </c>
-      <c r="G65" s="2" t="s">
+      <c r="H65" s="2" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>275</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C66" s="2" t="s">
+      <c r="C66" s="5" t="s">
         <v>277</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="E66" s="2" t="s">
+      <c r="E66" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="F66" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F66" s="3">
+      <c r="G66" s="3">
         <v>4300000</v>
       </c>
-      <c r="G66" s="2" t="s">
+      <c r="H66" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>280</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="C67" s="5" t="s">
         <v>282</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="E67" s="2" t="s">
+      <c r="E67" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="F67" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F67" s="3">
+      <c r="G67" s="3">
         <v>7900000</v>
       </c>
-      <c r="G67" s="2" t="s">
+      <c r="H67" s="2" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>285</v>
       </c>
@@ -3261,17 +3502,20 @@
       <c r="D68" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="E68" s="2" t="s">
+      <c r="E68" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="F68" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F68" s="3">
+      <c r="G68" s="3">
         <v>8800000</v>
       </c>
-      <c r="G68" s="2" t="s">
+      <c r="H68" s="2" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>290</v>
       </c>
@@ -3284,17 +3528,20 @@
       <c r="D69" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="E69" s="2" t="s">
+      <c r="E69" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F69" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F69" s="3">
+      <c r="G69" s="3">
         <v>4300000</v>
       </c>
-      <c r="G69" s="2" t="s">
+      <c r="H69" s="2" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>294</v>
       </c>
@@ -3307,17 +3554,20 @@
       <c r="D70" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="E70" s="2" t="s">
+      <c r="E70" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="F70" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F70" s="3">
+      <c r="G70" s="3">
         <v>4500000</v>
       </c>
-      <c r="G70" s="2" t="s">
+      <c r="H70" s="2" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>298</v>
       </c>
@@ -3330,17 +3580,20 @@
       <c r="D71" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="E71" s="2" t="s">
+      <c r="E71" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F71" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F71" s="3">
+      <c r="G71" s="3">
         <v>7200000</v>
       </c>
-      <c r="G71" s="2" t="s">
+      <c r="H71" s="2" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>302</v>
       </c>
@@ -3353,17 +3606,20 @@
       <c r="D72" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="E72" s="2" t="s">
+      <c r="E72" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="F72" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="F72" s="3">
+      <c r="G72" s="3">
         <v>1600000</v>
       </c>
-      <c r="G72" s="2" t="s">
+      <c r="H72" s="2" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>307</v>
       </c>
@@ -3376,17 +3632,20 @@
       <c r="D73" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="E73" s="2" t="s">
+      <c r="E73" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F73" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="F73" s="3">
+      <c r="G73" s="3">
         <v>1080000</v>
       </c>
-      <c r="G73" s="2" t="s">
+      <c r="H73" s="2" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>311</v>
       </c>
@@ -3399,17 +3658,20 @@
       <c r="D74" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="E74" s="2" t="s">
+      <c r="E74" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F74" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="F74" s="3">
+      <c r="G74" s="3">
         <v>2500000</v>
       </c>
-      <c r="G74" s="2" t="s">
+      <c r="H74" s="2" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>316</v>
       </c>
@@ -3422,17 +3684,20 @@
       <c r="D75" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="E75" s="2" t="s">
+      <c r="E75" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F75" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="F75" s="3">
+      <c r="G75" s="3">
         <v>900000</v>
       </c>
-      <c r="G75" s="2" t="s">
+      <c r="H75" s="2" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>320</v>
       </c>
@@ -3445,17 +3710,20 @@
       <c r="D76" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="E76" s="2" t="s">
+      <c r="E76" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F76" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="F76" s="3">
+      <c r="G76" s="3">
         <v>500000</v>
       </c>
-      <c r="G76" s="2" t="s">
+      <c r="H76" s="2" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>325</v>
       </c>
@@ -3468,17 +3736,20 @@
       <c r="D77" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="E77" s="2" t="s">
+      <c r="E77" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="F77" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="F77" s="3">
+      <c r="G77" s="3">
         <v>2300000</v>
       </c>
-      <c r="G77" s="2" t="s">
+      <c r="H77" s="2" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>330</v>
       </c>
@@ -3491,17 +3762,20 @@
       <c r="D78" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="E78" s="2" t="s">
+      <c r="E78" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F78" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="F78" s="3">
+      <c r="G78" s="3">
         <v>1620000</v>
       </c>
-      <c r="G78" s="2" t="s">
+      <c r="H78" s="2" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>334</v>
       </c>
@@ -3514,17 +3788,20 @@
       <c r="D79" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="E79" s="2" t="s">
+      <c r="E79" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F79" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="F79" s="3">
+      <c r="G79" s="3">
         <v>1780000</v>
       </c>
-      <c r="G79" s="2" t="s">
+      <c r="H79" s="2" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>338</v>
       </c>
@@ -3537,17 +3814,20 @@
       <c r="D80" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="E80" s="2" t="s">
+      <c r="E80" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F80" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="F80" s="3">
+      <c r="G80" s="3">
         <v>2600000</v>
       </c>
-      <c r="G80" s="2" t="s">
+      <c r="H80" s="2" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>342</v>
       </c>
@@ -3560,17 +3840,20 @@
       <c r="D81" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="E81" s="2" t="s">
+      <c r="E81" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F81" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="F81" s="3">
+      <c r="G81" s="3">
         <v>2380000</v>
       </c>
-      <c r="G81" s="2" t="s">
+      <c r="H81" s="2" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>346</v>
       </c>
@@ -3583,17 +3866,20 @@
       <c r="D82" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="E82" s="2" t="s">
+      <c r="E82" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F82" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="F82" s="3">
+      <c r="G82" s="3">
         <v>2700000</v>
       </c>
-      <c r="G82" s="2" t="s">
+      <c r="H82" s="2" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>351</v>
       </c>
@@ -3606,17 +3892,20 @@
       <c r="D83" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="E83" s="2" t="s">
+      <c r="E83" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="F83" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="F83" s="3">
+      <c r="G83" s="3">
         <v>3040000</v>
       </c>
-      <c r="G83" s="2" t="s">
+      <c r="H83" s="2" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>356</v>
       </c>
@@ -3629,17 +3918,20 @@
       <c r="D84" s="2" t="s">
         <v>358</v>
       </c>
-      <c r="E84" s="2" t="s">
+      <c r="E84" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F84" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="F84" s="3">
+      <c r="G84" s="3">
         <v>3660000</v>
       </c>
-      <c r="G84" s="2" t="s">
+      <c r="H84" s="2" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>360</v>
       </c>
@@ -3652,17 +3944,20 @@
       <c r="D85" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="E85" s="2" t="s">
+      <c r="E85" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F85" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="F85" s="3">
+      <c r="G85" s="3">
         <v>2740000</v>
       </c>
-      <c r="G85" s="2" t="s">
+      <c r="H85" s="2" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>364</v>
       </c>
@@ -3675,17 +3970,20 @@
       <c r="D86" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="E86" s="2" t="s">
+      <c r="E86" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F86" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="F86" s="3">
+      <c r="G86" s="3">
         <v>2300000</v>
       </c>
-      <c r="G86" s="2" t="s">
+      <c r="H86" s="2" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>368</v>
       </c>
@@ -3698,17 +3996,20 @@
       <c r="D87" s="2" t="s">
         <v>370</v>
       </c>
-      <c r="E87" s="2" t="s">
+      <c r="E87" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F87" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="F87" s="3">
+      <c r="G87" s="3">
         <v>3000000</v>
       </c>
-      <c r="G87" s="2" t="s">
+      <c r="H87" s="2" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>372</v>
       </c>
@@ -3721,17 +4022,20 @@
       <c r="D88" s="2" t="s">
         <v>374</v>
       </c>
-      <c r="E88" s="2" t="s">
+      <c r="E88" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F88" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="F88" s="3">
+      <c r="G88" s="3">
         <v>2600000</v>
       </c>
-      <c r="G88" s="2" t="s">
+      <c r="H88" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>376</v>
       </c>
@@ -3744,17 +4048,20 @@
       <c r="D89" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="E89" s="2" t="s">
+      <c r="E89" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F89" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="F89" s="3">
+      <c r="G89" s="3">
         <v>3100000</v>
       </c>
-      <c r="G89" s="2" t="s">
+      <c r="H89" s="2" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>380</v>
       </c>
@@ -3767,17 +4074,20 @@
       <c r="D90" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="E90" s="2" t="s">
+      <c r="E90" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F90" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="F90" s="3">
+      <c r="G90" s="3">
         <v>3060000</v>
       </c>
-      <c r="G90" s="2" t="s">
+      <c r="H90" s="2" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>384</v>
       </c>
@@ -3790,63 +4100,72 @@
       <c r="D91" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="E91" s="2" t="s">
+      <c r="E91" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="F91" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="F91" s="3">
+      <c r="G91" s="3">
         <v>3060000</v>
       </c>
-      <c r="G91" s="2" t="s">
+      <c r="H91" s="2" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>388</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="C92" s="2" t="s">
+      <c r="C92" s="5" t="s">
         <v>390</v>
       </c>
       <c r="D92" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="E92" s="2" t="s">
+      <c r="E92" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F92" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="F92" s="3">
+      <c r="G92" s="3">
         <v>9100000</v>
       </c>
-      <c r="G92" s="2" t="s">
+      <c r="H92" s="2" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>394</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="C93" s="2" t="s">
+      <c r="C93" s="5" t="s">
         <v>396</v>
       </c>
       <c r="D93" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="E93" s="2" t="s">
+      <c r="E93" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="F93" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="F93" s="3">
+      <c r="G93" s="3">
         <v>9800000</v>
       </c>
-      <c r="G93" s="2" t="s">
+      <c r="H93" s="2" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
         <v>399</v>
       </c>
@@ -3859,17 +4178,20 @@
       <c r="D94" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="E94" s="2" t="s">
+      <c r="E94" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="F94" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="F94" s="3">
+      <c r="G94" s="3">
         <v>7100000</v>
       </c>
-      <c r="G94" s="2" t="s">
+      <c r="H94" s="2" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>403</v>
       </c>
@@ -3882,17 +4204,20 @@
       <c r="D95" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="E95" s="2" t="s">
+      <c r="E95" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F95" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="F95" s="3">
+      <c r="G95" s="3">
         <v>9000000</v>
       </c>
-      <c r="G95" s="2" t="s">
+      <c r="H95" s="2" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>407</v>
       </c>
@@ -3905,17 +4230,20 @@
       <c r="D96" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="E96" s="2" t="s">
+      <c r="E96" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="F96" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="F96" s="3">
+      <c r="G96" s="3">
         <v>10900000</v>
       </c>
-      <c r="G96" s="2" t="s">
+      <c r="H96" s="2" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>411</v>
       </c>
@@ -3928,17 +4256,20 @@
       <c r="D97" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="E97" s="2" t="s">
+      <c r="E97" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F97" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="F97" s="3">
+      <c r="G97" s="3">
         <v>11600000</v>
       </c>
-      <c r="G97" s="2" t="s">
+      <c r="H97" s="2" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>415</v>
       </c>
@@ -3951,17 +4282,20 @@
       <c r="D98" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="E98" s="2" t="s">
+      <c r="E98" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="F98" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="F98" s="3">
+      <c r="G98" s="3">
         <v>10100000</v>
       </c>
-      <c r="G98" s="2" t="s">
+      <c r="H98" s="2" t="s">
         <v>418</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
         <v>419</v>
       </c>
@@ -3974,79 +4308,89 @@
       <c r="D99" s="2" t="s">
         <v>421</v>
       </c>
-      <c r="E99" s="2" t="s">
+      <c r="E99" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="F99" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="F99" s="3">
+      <c r="G99" s="3">
         <v>8600000</v>
       </c>
-      <c r="G99" s="2" t="s">
+      <c r="H99" s="2" t="s">
         <v>422</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>423</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="C100" s="2" t="s">
+      <c r="C100" s="5" t="s">
         <v>282</v>
       </c>
       <c r="D100" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="E100" s="2" t="s">
+      <c r="E100" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="F100" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="F100" s="3">
+      <c r="G100" s="3">
         <v>9900000</v>
       </c>
-      <c r="G100" s="2" t="s">
+      <c r="H100" s="2" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>427</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="C101" s="2" t="s">
+      <c r="C101" s="5" t="s">
         <v>47</v>
       </c>
       <c r="D101" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="E101" s="2" t="s">
+      <c r="E101" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="F101" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="F101" s="3">
+      <c r="G101" s="3">
         <v>6100000</v>
       </c>
-      <c r="G101" s="2" t="s">
+      <c r="H101" s="2" t="s">
         <v>430</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G101" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H101" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="4" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>2</v>
       </c>
@@ -4060,7 +4404,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -4074,7 +4418,7 @@
         <v>22800000</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>75</v>
       </c>
@@ -4088,7 +4432,7 @@
         <v>15300000</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>136</v>
       </c>
@@ -4102,7 +4446,7 @@
         <v>17800000</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>218</v>
       </c>
@@ -4116,7 +4460,7 @@
         <v>18000000</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>261</v>
       </c>
@@ -4130,7 +4474,7 @@
         <v>8800000</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>305</v>
       </c>
@@ -4144,7 +4488,7 @@
         <v>2600000</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>349</v>
       </c>
@@ -4158,7 +4502,7 @@
         <v>3660000</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>392</v>
       </c>

</xml_diff>